<commit_message>
Restructure projet : arborescence V2, README, archivage des fichiers V1 obsolètes
</commit_message>
<xml_diff>
--- a/docs/PPMT_Arborescence_Issue_Tree_V2.xlsx
+++ b/docs/PPMT_Arborescence_Issue_Tree_V2.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B3:B48"/>
+  <dimension ref="B3:B52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -545,119 +545,119 @@
     <row r="11">
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>│   ├── ppmt.db                # Base SQLite : 62 435 offres, 1 514 métiers ROME (fournie par data_ppmt_octobre.zip)</t>
+          <t>│   ├── offres_ft_idf.csv      # France Travail aplati, produit par collect.py (entrée de prepare.py)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>│   ├── ml_resultats.json      # Résultats du Machine Learning (AUC, F1, variables importantes)</t>
+          <t>│   ├── offres_idf.csv         # Adzuna aplati, produit par collect.py (entrée de prepare.py)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>│   └── predictions_tension.csv# Prédictions « en tension » par métier</t>
+          <t>│   ├── offres_ft_idf_clean.csv  # Version nettoyée de secours, versionnée dans Git (lue si les bruts sont absents)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>│</t>
+          <t>│   ├── offres_idf_clean.csv   # Idem pour Adzuna</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>├── logs/                      # collect_AAAAMMJJ_HHMMSS.log : un journal horodaté par collecte</t>
+          <t>│   ├── ppmt.db                # Base SQLite : 62 435 offres, 1 514 métiers ROME (fournie par data_ppmt_octobre.zip)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>│</t>
+          <t>│   ├── ml_resultats.json      # Résultats du Machine Learning (AUC, F1, variables importantes)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>├── notebook/                  # Espace d'expérimentation</t>
+          <t>│   └── predictions_tension.csv# Prédictions « en tension » par métier</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>│   └── ml_tests.py            # ML V2 : classification « en tension » (XGBoost, AUC 0,886)</t>
+          <t>│</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>│</t>
+          <t>├── logs/                      # collect_AAAAMMJJ_HHMMSS.log : un journal horodaté par collecte</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>├── src/                       # Le cœur logique : scripts Python permanents du pipeline (ex-« sources/ »)</t>
+          <t>│</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>│   ├── collect.py             # C1 : France Travail (OAuth2, cascade), Adzuna, contours et communes IDF</t>
+          <t>├── notebook/                  # Espace d'expérimentation</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>│   ├── prepare.py             # C2/C3 : nettoyage, dédoublonnage, salaires, codes ROME, RGPD</t>
+          <t>│   └── ml_tests.py            # ML V2 : classification « en tension » (XGBoost, AUC 0,886)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>│   └── store.py               # C4 : schéma SQLite, chargement, agrégation SQL, purge 12 mois</t>
+          <t>│</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>│</t>
+          <t>├── src/                       # Le cœur logique : scripts Python permanents du pipeline (ex-« sources/ »)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>├── api/</t>
+          <t>│   ├── collect.py             # C1 : France Travail (OAuth2, cascade), Adzuna, contours et communes IDF</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>│   ├── main.py                # C5 : API REST FastAPI (7 routes, clé X-API-Key, Swagger)</t>
+          <t>│   ├── prepare.py             # C2/C3 : nettoyage, dédoublonnage, salaires, codes ROME, RGPD</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>│   └── requirements-api.txt   # Dépendances de l'API seule (image Docker allégée)</t>
+          <t>│   └── store.py               # C4 : schéma SQLite, chargement, agrégation SQL, purge 12 mois</t>
         </is>
       </c>
     </row>
@@ -671,21 +671,21 @@
     <row r="29">
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>├── webapp/                    # Interface utilisateur (ce que le jury manipule)</t>
+          <t>├── api/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>│   ├── app.py                 # Dashboard Streamlit : 6 onglets, lit data/ppmt.db</t>
+          <t>│   ├── main.py                # C5 : API REST FastAPI (7 routes, clé X-API-Key, Swagger)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>│   └── models/                # Modèles ML sauvegardés, utilisés par le dashboard</t>
+          <t>│   └── requirements-api.txt   # Dépendances de l'API seule (image Docker allégée)</t>
         </is>
       </c>
     </row>
@@ -699,110 +699,138 @@
     <row r="33">
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>├── tests/</t>
+          <t>├── webapp/                    # Interface utilisateur (ce que le jury manipule)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>│   └── test_pipeline.py       # 57 tests pytest (collecte simulée, règles, base, API)</t>
+          <t>│   ├── app.py                 # Dashboard Streamlit : 6 onglets, lit data/ppmt.db</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>│</t>
+          <t>│   └── models/                # Modèles ML sauvegardés, utilisés par le dashboard</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>├── docs/</t>
+          <t>│</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>│   ├── dictionnaire.md        # Dictionnaire de données</t>
+          <t>├── tests/</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>│   ├── rgpd.md                # Registre des traitements RGPD</t>
+          <t>│   └── test_pipeline.py       # 57 tests pytest (collecte simulée, règles, base, API)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>│   ├── arborescence.md        # Ce plan commenté</t>
+          <t>│</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>│   ├── issue_tree.md          # Issue Tree du projet</t>
+          <t>├── docs/</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>│   └── PPMT_Arborescence_Issue_Tree_V2.xlsx   # Classeur de cadrage (arborescence, explications, Issue Tree)</t>
+          <t>│   ├── dictionnaire.md        # Dictionnaire de données</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>│</t>
+          <t>│   ├── rgpd.md                # Registre des traitements RGPD</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>├── run_pipeline.py            # Orchestrateur C1 → C4 (python run_pipeline.py --collect)</t>
+          <t>│   ├── arborescence.md        # Ce plan commenté</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>├── Dockerfile                 # Image de l'API</t>
+          <t>│   ├── issue_tree.md          # Issue Tree du projet</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>├── .env.example               # Noms des variables d'environnement (jamais de valeurs)</t>
+          <t>│   └── PPMT_Arborescence_Issue_Tree_V2.xlsx   # Classeur de cadrage (arborescence, explications, Issue Tree)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>├── .gitignore                 # Ignore .env, data/raw/, environnements Python</t>
+          <t>│</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>├── requirements.txt           # Outils Python à installer (pip install -r requirements.txt)</t>
+          <t>├── run_pipeline.py            # Orchestrateur C1 → C4 (python run_pipeline.py --collect)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>├── Dockerfile                 # Image de l'API</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>├── .env.example               # Noms des variables d'environnement (jamais de valeurs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>├── .gitignore                 # Ignore .env, data/raw/, environnements Python</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>├── requirements.txt           # Outils Python à installer (pip install -r requirements.txt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="3" t="inlineStr">
         <is>
           <t>└── README.md                  # Page d'accueil GitHub : notice, Issue Tree, dictionnaire de données</t>
         </is>
@@ -820,7 +848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B3:B60"/>
+  <dimension ref="B3:B62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -862,204 +890,211 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1">
+    <row r="12" ht="43.5" customHeight="1">
       <c r="B12" s="5" t="inlineStr">
         <is>
+          <t>offres_ft_idf.csv et offres_idf.csv : les offres aplaties (une ligne par offre) que collect.py écrit à partir des réponses brutes ; c'est l'entrée de prepare.py. offres_ft_idf_clean.csv et offres_idf_clean.csv sont des versions nettoyées de secours, versionnées dans Git : prepare.py les lit si les fichiers bruts sont absents.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="B14" s="5" t="inlineStr">
+        <is>
           <t>ppmt.db, ml_resultats.json, predictions_tension.csv : la base SQLite (62 435 offres) et les résultats du Machine Learning. Pour la soutenance, la base est figée au 6 octobre 2026 : elle est fournie par l'archive data_ppmt_octobre.zip.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="43.5" customHeight="1">
-      <c r="B14" s="5" t="inlineStr">
+    <row r="16" ht="43.5" customHeight="1">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>⚠️ Pourquoi le .gitignore ? Les fichiers bruts pèsent lourd, contiennent des données non masquées, et ne doivent jamais être publiés. Le .gitignore ordonne à Git : « suis mon code, mais ne touche pas à data/raw/ ». Le fichier .env (identifiants) est ignoré pour la même raison.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="B16" s="4" t="inlineStr">
+    <row r="18" ht="22" customHeight="1">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>🧾 2. Le dossier logs/ : le journal de bord</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="B17" s="5" t="inlineStr">
+    <row r="19" ht="30" customHeight="1">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Chaque collecte écrit un journal horodaté (collect_AAAAMMJJ_HHMMSS.log) : zones découpées, avertissements, bilan de couverture (63 173 offres sur 63 504 annoncées le 6 octobre). C'est la preuve de ce que la collecte a réellement fait.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="B19" s="4" t="inlineStr">
+    <row r="21" ht="22" customHeight="1">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>📓 3. Le dossier notebook/ : le laboratoire d'expérimentation</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="B20" s="5" t="inlineStr">
+    <row r="22" ht="30" customHeight="1">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>ml_tests.py : l'expérimentation Machine Learning de la V2. La V1 annonçait un R² de 0,995, dû à une fuite de données ; la V2 classe les 717 métiers d'au moins 10 offres en « en tension » ou non (XGBoost : AUC 0,886, F1 0,785). Hors du bloc BC01, c'est une ouverture.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="B22" s="4" t="inlineStr">
+    <row r="24" ht="22" customHeight="1">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>🛠️ 4. Le dossier src/ : les machines automatisées de l'usine</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="B23" s="5" t="inlineStr">
+    <row r="25" ht="30" customHeight="1">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>C'est le dossier le plus important pour l'évaluation du bloc (le pipeline). Ce sont des scripts Python permanents, chacun testable et exécutable seul. Il remplace le dossier « sources/ » du plan de mai : même rôle, nom plus courant.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="57" customHeight="1">
-      <c r="B25" s="5" t="inlineStr">
+    <row r="27" ht="57" customHeight="1">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>collect.py (la pompe à API) : se connecte à France Travail en OAuth2 (client_credentials), renouvelle le jeton toutes les 20 minutes, et télécharge les offres. L'API plafonne à 3 150 offres par requête : la collecte découpe en cascade (département, fenêtres de dates, type de contrat). Il lit aussi Adzuna (échantillon de 12 500 offres sur 220 238), les contours des départements et les 1 276 communes d'Île-de-France. 3 tentatives avec attente croissante, pause de 100 ms entre deux appels.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="43.5" customHeight="1">
-      <c r="B27" s="5" t="inlineStr">
+    <row r="29" ht="43.5" customHeight="1">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>prepare.py (le centre de tri) : prend les fichiers de data/raw/, supprime les doublons (URL, puis titre + entreprise + lieu), complète les salaires manquants par une médiane (56 % non affichés), rattache les offres Adzuna aux codes ROME, harmonise les contrats en 7 catégories, masque les e-mails et téléphones (RGPD).</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="B29" s="5" t="inlineStr">
+    <row r="31" ht="30" customHeight="1">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>store.py (le rangement) : crée le schéma SQLite (4 tables, clés étrangères, contraintes CHECK/UNIQUE, 6 index), charge les offres, calcule les indicateurs de tension en SQL, purge les offres de plus de 12 mois. C'est l'équivalent du schema_db.sql du plan de mai.</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="B31" s="4" t="inlineStr">
+    <row r="33" ht="22" customHeight="1">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>🌐 5. Le dossier api/ : la porte d'entrée pour les développeurs</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="43.5" customHeight="1">
-      <c r="B32" s="5" t="inlineStr">
+    <row r="34" ht="43.5" customHeight="1">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>main.py : l'API FastAPI. requirements-api.txt liste ses seules dépendances, pour une image Docker légère. 7 routes en lecture seule, protégées par une clé X-API-Key (403 sans clé), paramètres validés par Pydantic (422), SQL paramétré, base ouverte en lecture seule. La documentation interactive (Swagger) est sur /docs.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="22" customHeight="1">
-      <c r="B34" s="4" t="inlineStr">
+    <row r="36" ht="22" customHeight="1">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>💻 6. Le dossier webapp/ : la vitrine du magasin</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="43.5" customHeight="1">
-      <c r="B35" s="5" t="inlineStr">
+    <row r="37" ht="43.5" customHeight="1">
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>app.py : le dashboard Streamlit (6 onglets, filtres par département, contrat et secteur). Il ne collecte rien : il lit uniquement data/ppmt.db. models/ contient les modèles ML sauvegardés. Une version en ligne sert de secours : https://ppmt-claire.streamlit.app (branche demo-cloud).</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="22" customHeight="1">
-      <c r="B37" s="4" t="inlineStr">
+    <row r="39" ht="22" customHeight="1">
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>✅ 7. Le dossier tests/ : le contrôle qualité</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="B38" s="5" t="inlineStr">
+    <row r="40" ht="30" customHeight="1">
+      <c r="B40" s="5" t="inlineStr">
         <is>
           <t>test_pipeline.py : 57 tests pytest. 4 pour la collecte (API simulées), 31 pour les règles de préparation, 13 pour la base, 9 pour l'API. Limite connue : la cascade France Travail n'a pas encore de test unitaire dédié.</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="22" customHeight="1">
-      <c r="B40" s="4" t="inlineStr">
+    <row r="42" ht="22" customHeight="1">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>📄 8. Les fichiers à la racine (les indispensables de gestion)</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="16.5" customHeight="1">
-      <c r="B41" s="5" t="inlineStr">
+    <row r="43" ht="16.5" customHeight="1">
+      <c r="B43" s="5" t="inlineStr">
         <is>
           <t>README.md : la notice du projet : problème, Issue Tree, arborescence, dictionnaire de données, lancement, API, limites.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="30" customHeight="1">
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>requirements.txt : la liste des outils Python. Une seule commande (pip install -r requirements.txt) installe les mêmes versions chez tout le monde.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="30" customHeight="1">
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>.env.example : la liste des variables d'environnement attendues (identifiants France Travail et Adzuna), sans aucune valeur. On le copie en .env, qui n'est jamais envoyé sur Git.</t>
+          <t>requirements.txt : la liste des outils Python. Une seule commande (pip install -r requirements.txt) installe les mêmes versions chez tout le monde.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="30" customHeight="1">
       <c r="B47" s="5" t="inlineStr">
         <is>
+          <t>.env.example : la liste des variables d'environnement attendues (identifiants France Travail et Adzuna), sans aucune valeur. On le copie en .env, qui n'est jamais envoyé sur Git.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="B49" s="5" t="inlineStr">
+        <is>
           <t>run_pipeline.py : l'orchestrateur. Il enchaîne la collecte, la préparation et le stockage ; sans l'option --collect, il repart des fichiers bruts déjà présents dans data/raw/.</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1">
-      <c r="B49" s="5" t="inlineStr">
+    <row r="51" ht="16.5" customHeight="1">
+      <c r="B51" s="5" t="inlineStr">
         <is>
           <t>Dockerfile : l'image de l'API (FastAPI, Uvicorn et Pydantic seulement), déployable sur Google Cloud Run ou Render.</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="22" customHeight="1">
-      <c r="B51" s="4" t="inlineStr">
+    <row r="53" ht="22" customHeight="1">
+      <c r="B53" s="4" t="inlineStr">
         <is>
           <t>💡 En résumé, comment les données circulent dans cette structure :</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="16.5" customHeight="1">
-      <c r="B52" s="5" t="inlineStr">
-        <is>
-          <t>1. collect.py télécharge les données dans data/raw/ (et écrit son journal dans logs/).</t>
         </is>
       </c>
     </row>
     <row r="54" ht="16.5" customHeight="1">
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>2. prepare.py nettoie le tout et écrit data/processed/offres_unifiees.csv.</t>
+          <t>1. collect.py télécharge les données dans data/raw/ (et écrit son journal dans logs/).</t>
         </is>
       </c>
     </row>
     <row r="56" ht="16.5" customHeight="1">
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>3. store.py range les offres dans la base SQLite data/ppmt.db et calcule les indicateurs de tension.</t>
+          <t>2. prepare.py nettoie le tout et écrit data/processed/offres_unifiees.csv.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="16.5" customHeight="1">
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>4. api/main.py et webapp/app.py lisent cette base : l'API pour les développeurs, le dashboard pour les utilisateurs.</t>
+          <t>3. store.py range les offres dans la base SQLite data/ppmt.db et calcule les indicateurs de tension.</t>
         </is>
       </c>
     </row>
     <row r="60" ht="16.5" customHeight="1">
       <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>4. api/main.py et webapp/app.py lisent cette base : l'API pour les développeurs, le dashboard pour les utilisateurs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="16.5" customHeight="1">
+      <c r="B62" s="5" t="inlineStr">
         <is>
           <t>5. tests/ vérifie chaque étape ; notebook/ml_tests.py ajoute le modèle de classification des métiers en tension.</t>
         </is>

</xml_diff>

<commit_message>
docs : pytest.ini ajouté à l'arborescence
</commit_message>
<xml_diff>
--- a/docs/PPMT_Arborescence_Issue_Tree_V2.xlsx
+++ b/docs/PPMT_Arborescence_Issue_Tree_V2.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B3:B52"/>
+  <dimension ref="B3:B53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -818,19 +818,26 @@
     <row r="50">
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>├── .gitignore                 # Ignore .env, data/raw/, environnements Python</t>
+          <t>├── .gitignore                 # Ignore .env, data/raw/, _archive/, caches Python et pytest, .vscode/</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>├── requirements.txt           # Outils Python à installer (pip install -r requirements.txt)</t>
+          <t>├── pytest.ini                 # Réglages de pytest : dossier des tests, cache rangé dans zz_pytest_cache/</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>├── requirements.txt           # Outils Python à installer (pip install -r requirements.txt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>└── README.md                  # Page d'accueil GitHub : notice, Issue Tree, dictionnaire de données</t>
         </is>
@@ -848,7 +855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B3:B62"/>
+  <dimension ref="B3:B64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1033,68 +1040,75 @@
     <row r="45" ht="30" customHeight="1">
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>requirements.txt : la liste des outils Python. Une seule commande (pip install -r requirements.txt) installe les mêmes versions chez tout le monde.</t>
+          <t>pytest.ini : les réglages de pytest, l'outil qui lance les 57 tests. Il indique où sont les tests (tests/) et range le cache de pytest dans zz_pytest_cache/, un dossier ignoré par Git qui s'affiche en bas de l'explorateur. Il suffit alors de taper pytest -q.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="30" customHeight="1">
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>.env.example : la liste des variables d'environnement attendues (identifiants France Travail et Adzuna), sans aucune valeur. On le copie en .env, qui n'est jamais envoyé sur Git.</t>
+          <t>requirements.txt : la liste des outils Python. Une seule commande (pip install -r requirements.txt) installe les mêmes versions chez tout le monde.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="30" customHeight="1">
       <c r="B49" s="5" t="inlineStr">
         <is>
+          <t>.env.example : la liste des variables d'environnement attendues (identifiants France Travail et Adzuna), sans aucune valeur. On le copie en .env, qui n'est jamais envoyé sur Git.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="B51" s="5" t="inlineStr">
+        <is>
           <t>run_pipeline.py : l'orchestrateur. Il enchaîne la collecte, la préparation et le stockage ; sans l'option --collect, il repart des fichiers bruts déjà présents dans data/raw/.</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="16.5" customHeight="1">
-      <c r="B51" s="5" t="inlineStr">
+    <row r="53" ht="16.5" customHeight="1">
+      <c r="B53" s="5" t="inlineStr">
         <is>
           <t>Dockerfile : l'image de l'API (FastAPI, Uvicorn et Pydantic seulement), déployable sur Google Cloud Run ou Render.</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="22" customHeight="1">
-      <c r="B53" s="4" t="inlineStr">
+    <row r="55" ht="22" customHeight="1">
+      <c r="B55" s="4" t="inlineStr">
         <is>
           <t>💡 En résumé, comment les données circulent dans cette structure :</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="16.5" customHeight="1">
-      <c r="B54" s="5" t="inlineStr">
-        <is>
-          <t>1. collect.py télécharge les données dans data/raw/ (et écrit son journal dans logs/).</t>
         </is>
       </c>
     </row>
     <row r="56" ht="16.5" customHeight="1">
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>2. prepare.py nettoie le tout et écrit data/processed/offres_unifiees.csv.</t>
+          <t>1. collect.py télécharge les données dans data/raw/ (et écrit son journal dans logs/).</t>
         </is>
       </c>
     </row>
     <row r="58" ht="16.5" customHeight="1">
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>3. store.py range les offres dans la base SQLite data/ppmt.db et calcule les indicateurs de tension.</t>
+          <t>2. prepare.py nettoie le tout et écrit data/processed/offres_unifiees.csv.</t>
         </is>
       </c>
     </row>
     <row r="60" ht="16.5" customHeight="1">
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>4. api/main.py et webapp/app.py lisent cette base : l'API pour les développeurs, le dashboard pour les utilisateurs.</t>
+          <t>3. store.py range les offres dans la base SQLite data/ppmt.db et calcule les indicateurs de tension.</t>
         </is>
       </c>
     </row>
     <row r="62" ht="16.5" customHeight="1">
       <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>4. api/main.py et webapp/app.py lisent cette base : l'API pour les développeurs, le dashboard pour les utilisateurs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="16.5" customHeight="1">
+      <c r="B64" s="5" t="inlineStr">
         <is>
           <t>5. tests/ vérifie chaque étape ; notebook/ml_tests.py ajoute le modèle de classification des métiers en tension.</t>
         </is>

</xml_diff>

<commit_message>
docs : dossier, diaporama et documents d'octobre
</commit_message>
<xml_diff>
--- a/docs/PPMT_Arborescence_Issue_Tree_V2.xlsx
+++ b/docs/PPMT_Arborescence_Issue_Tree_V2.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B3:B53"/>
+  <dimension ref="B3:B54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -755,89 +755,96 @@
     <row r="41">
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>│   ├── dictionnaire.md        # Dictionnaire de données</t>
+          <t>│   ├── soutenance/            # Documents de la soutenance du 16 octobre : dossier (Word, PDF), diaporama, fiche technique V1/V2</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>│   ├── rgpd.md                # Registre des traitements RGPD</t>
+          <t>│   ├── dictionnaire.md        # Dictionnaire de données</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>│   ├── arborescence.md        # Ce plan commenté</t>
+          <t>│   ├── rgpd.md                # Registre des traitements RGPD</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>│   ├── issue_tree.md          # Issue Tree du projet</t>
+          <t>│   ├── arborescence.md        # Ce plan commenté</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>│   └── PPMT_Arborescence_Issue_Tree_V2.xlsx   # Classeur de cadrage (arborescence, explications, Issue Tree)</t>
+          <t>│   ├── issue_tree.md          # Issue Tree du projet</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>│</t>
+          <t>│   └── PPMT_Arborescence_Issue_Tree_V2.xlsx   # Classeur de cadrage (arborescence, explications, Issue Tree)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>├── run_pipeline.py            # Orchestrateur C1 → C4 (python run_pipeline.py --collect)</t>
+          <t>│</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>├── Dockerfile                 # Image de l'API</t>
+          <t>├── run_pipeline.py            # Orchestrateur C1 → C4 (python run_pipeline.py --collect)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>├── .env.example               # Noms des variables d'environnement (jamais de valeurs)</t>
+          <t>├── Dockerfile                 # Image de l'API</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>├── .gitignore                 # Ignore .env, data/raw/, _archive/, caches Python et pytest, .vscode/</t>
+          <t>├── .env.example               # Noms des variables d'environnement (jamais de valeurs)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>├── pytest.ini                 # Réglages de pytest : dossier des tests, cache rangé dans zz_pytest_cache/</t>
+          <t>├── .gitignore                 # Ignore .env, data/raw/, _archive/, caches Python et pytest, .vscode/</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>├── requirements.txt           # Outils Python à installer (pip install -r requirements.txt)</t>
+          <t>├── pytest.ini                 # Réglages de pytest : dossier des tests, cache rangé dans zz_pytest_cache/</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>├── requirements.txt           # Outils Python à installer (pip install -r requirements.txt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="3" t="inlineStr">
         <is>
           <t>└── README.md                  # Page d'accueil GitHub : notice, Issue Tree, dictionnaire de données</t>
         </is>
@@ -855,7 +862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B3:B64"/>
+  <dimension ref="B3:B69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -946,169 +953,190 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="B24" s="4" t="inlineStr">
+    <row r="24" ht="70.5" customHeight="1">
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Comment sont construites les prédictions : la cible est « indice de tension &gt; 100 » (46 % des 717 métiers) ; les variables d'entrée décrivent le profil des offres du métier (parts de CDI, CDD et intérim, salaire, part de salaires non affichés, expérience demandée, part d'offres pour débutants, longueur des descriptions, famille ROME), sans aucune variable de volume. Chaque probabilité de predictions_tension.csv (colonne proba_tension) est prédite en validation croisée à 5 plis : le métier est prédit par un modèle qui ne l'a pas vu à l'entraînement. Sans la longueur des descriptions, l'AUC de XGBoost passe de 0,886 à 0,795.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>🛠️ 4. Le dossier src/ : les machines automatisées de l'usine</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="B25" s="5" t="inlineStr">
+    <row r="27" ht="30" customHeight="1">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>C'est le dossier le plus important pour l'évaluation du bloc (le pipeline). Ce sont des scripts Python permanents, chacun testable et exécutable seul. Il remplace le dossier « sources/ » du plan de mai : même rôle, nom plus courant.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="57" customHeight="1">
-      <c r="B27" s="5" t="inlineStr">
+    <row r="29" ht="57" customHeight="1">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>collect.py (la pompe à API) : se connecte à France Travail en OAuth2 (client_credentials), renouvelle le jeton toutes les 20 minutes, et télécharge les offres. L'API plafonne à 3 150 offres par requête : la collecte découpe en cascade (département, fenêtres de dates, type de contrat). Il lit aussi Adzuna (échantillon de 12 500 offres sur 220 238), les contours des départements et les 1 276 communes d'Île-de-France. 3 tentatives avec attente croissante, pause de 100 ms entre deux appels.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="43.5" customHeight="1">
-      <c r="B29" s="5" t="inlineStr">
+    <row r="31" ht="43.5" customHeight="1">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>prepare.py (le centre de tri) : prend les fichiers de data/raw/, supprime les doublons (URL, puis titre + entreprise + lieu), complète les salaires manquants par une médiane (56 % non affichés), rattache les offres Adzuna aux codes ROME, harmonise les contrats en 7 catégories, masque les e-mails et téléphones (RGPD).</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="B31" s="5" t="inlineStr">
+    <row r="33" ht="30" customHeight="1">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>store.py (le rangement) : crée le schéma SQLite (4 tables, clés étrangères, contraintes CHECK/UNIQUE, 6 index), charge les offres, calcule les indicateurs de tension en SQL, purge les offres de plus de 12 mois. C'est l'équivalent du schema_db.sql du plan de mai.</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="22" customHeight="1">
-      <c r="B33" s="4" t="inlineStr">
+    <row r="35" ht="22" customHeight="1">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>🌐 5. Le dossier api/ : la porte d'entrée pour les développeurs</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="43.5" customHeight="1">
-      <c r="B34" s="5" t="inlineStr">
+    <row r="36" ht="43.5" customHeight="1">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>main.py : l'API FastAPI. requirements-api.txt liste ses seules dépendances, pour une image Docker légère. 7 routes en lecture seule, protégées par une clé X-API-Key (403 sans clé), paramètres validés par Pydantic (422), SQL paramétré, base ouverte en lecture seule. La documentation interactive (Swagger) est sur /docs.</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="22" customHeight="1">
-      <c r="B36" s="4" t="inlineStr">
+    <row r="38" ht="22" customHeight="1">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>💻 6. Le dossier webapp/ : la vitrine du magasin</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="43.5" customHeight="1">
-      <c r="B37" s="5" t="inlineStr">
+    <row r="39" ht="43.5" customHeight="1">
+      <c r="B39" s="5" t="inlineStr">
         <is>
           <t>app.py : le dashboard Streamlit (6 onglets, filtres par département, contrat et secteur). Il ne collecte rien : il lit uniquement data/ppmt.db. models/ contient les modèles ML sauvegardés. Une version en ligne sert de secours : https://ppmt-claire.streamlit.app (branche demo-cloud).</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="22" customHeight="1">
-      <c r="B39" s="4" t="inlineStr">
+    <row r="41" ht="22" customHeight="1">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>✅ 7. Le dossier tests/ : le contrôle qualité</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="30" customHeight="1">
-      <c r="B40" s="5" t="inlineStr">
+    <row r="42" ht="30" customHeight="1">
+      <c r="B42" s="5" t="inlineStr">
         <is>
           <t>test_pipeline.py : 57 tests pytest. 4 pour la collecte (API simulées), 31 pour les règles de préparation, 13 pour la base, 9 pour l'API. Limite connue : la cascade France Travail n'a pas encore de test unitaire dédié.</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="22" customHeight="1">
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>📄 8. Les fichiers à la racine (les indispensables de gestion)</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="16.5" customHeight="1">
-      <c r="B43" s="5" t="inlineStr">
+    <row r="44" ht="22" customHeight="1">
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>📚 8. Le dossier docs/ : la documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="43.5" customHeight="1">
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>dictionnaire.md (les données), rgpd.md (les traitements), arborescence.md (ce plan), issue_tree.md et le classeur PPMT_Arborescence_Issue_Tree_V2.xlsx. Le sous-dossier soutenance/ contient les documents de la soutenance du 16 octobre : dossier (Word et PDF), diaporama et fiche technique V1/V2. Les documents de la V1 ont été rangés hors du dépôt, dans _archive/.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>📄 9. Les fichiers à la racine (les indispensables de gestion)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="16.5" customHeight="1">
+      <c r="B48" s="5" t="inlineStr">
         <is>
           <t>README.md : la notice du projet : problème, Issue Tree, arborescence, dictionnaire de données, lancement, API, limites.</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="30" customHeight="1">
-      <c r="B45" s="5" t="inlineStr">
+    <row r="50" ht="30" customHeight="1">
+      <c r="B50" s="5" t="inlineStr">
         <is>
           <t>pytest.ini : les réglages de pytest, l'outil qui lance les 57 tests. Il indique où sont les tests (tests/) et range le cache de pytest dans zz_pytest_cache/, un dossier ignoré par Git qui s'affiche en bas de l'explorateur. Il suffit alors de taper pytest -q.</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="30" customHeight="1">
-      <c r="B47" s="5" t="inlineStr">
+    <row r="52" ht="30" customHeight="1">
+      <c r="B52" s="5" t="inlineStr">
         <is>
           <t>requirements.txt : la liste des outils Python. Une seule commande (pip install -r requirements.txt) installe les mêmes versions chez tout le monde.</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="30" customHeight="1">
-      <c r="B49" s="5" t="inlineStr">
+    <row r="54" ht="30" customHeight="1">
+      <c r="B54" s="5" t="inlineStr">
         <is>
           <t>.env.example : la liste des variables d'environnement attendues (identifiants France Travail et Adzuna), sans aucune valeur. On le copie en .env, qui n'est jamais envoyé sur Git.</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="30" customHeight="1">
-      <c r="B51" s="5" t="inlineStr">
+    <row r="56" ht="30" customHeight="1">
+      <c r="B56" s="5" t="inlineStr">
         <is>
           <t>run_pipeline.py : l'orchestrateur. Il enchaîne la collecte, la préparation et le stockage ; sans l'option --collect, il repart des fichiers bruts déjà présents dans data/raw/.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="16.5" customHeight="1">
-      <c r="B53" s="5" t="inlineStr">
-        <is>
-          <t>Dockerfile : l'image de l'API (FastAPI, Uvicorn et Pydantic seulement), déployable sur Google Cloud Run ou Render.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="22" customHeight="1">
-      <c r="B55" s="4" t="inlineStr">
-        <is>
-          <t>💡 En résumé, comment les données circulent dans cette structure :</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="16.5" customHeight="1">
-      <c r="B56" s="5" t="inlineStr">
-        <is>
-          <t>1. collect.py télécharge les données dans data/raw/ (et écrit son journal dans logs/).</t>
         </is>
       </c>
     </row>
     <row r="58" ht="16.5" customHeight="1">
       <c r="B58" s="5" t="inlineStr">
         <is>
+          <t>Dockerfile : l'image de l'API (FastAPI, Uvicorn et Pydantic seulement), déployable sur Google Cloud Run ou Render.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>💡 En résumé, comment les données circulent dans cette structure :</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="16.5" customHeight="1">
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>1. collect.py télécharge les données dans data/raw/ (et écrit son journal dans logs/).</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="16.5" customHeight="1">
+      <c r="B63" s="5" t="inlineStr">
+        <is>
           <t>2. prepare.py nettoie le tout et écrit data/processed/offres_unifiees.csv.</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="16.5" customHeight="1">
-      <c r="B60" s="5" t="inlineStr">
+    <row r="65" ht="16.5" customHeight="1">
+      <c r="B65" s="5" t="inlineStr">
         <is>
           <t>3. store.py range les offres dans la base SQLite data/ppmt.db et calcule les indicateurs de tension.</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="16.5" customHeight="1">
-      <c r="B62" s="5" t="inlineStr">
+    <row r="67" ht="16.5" customHeight="1">
+      <c r="B67" s="5" t="inlineStr">
         <is>
           <t>4. api/main.py et webapp/app.py lisent cette base : l'API pour les développeurs, le dashboard pour les utilisateurs.</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="16.5" customHeight="1">
-      <c r="B64" s="5" t="inlineStr">
+    <row r="69" ht="16.5" customHeight="1">
+      <c r="B69" s="5" t="inlineStr">
         <is>
           <t>5. tests/ vérifie chaque étape ; notebook/ml_tests.py ajoute le modèle de classification des métiers en tension.</t>
         </is>

</xml_diff>

<commit_message>
Met à jour README, arborescence et classeur : fiche V1/V2 retirée
</commit_message>
<xml_diff>
--- a/docs/PPMT_Arborescence_Issue_Tree_V2.xlsx
+++ b/docs/PPMT_Arborescence_Issue_Tree_V2.xlsx
@@ -755,7 +755,7 @@
     <row r="41">
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>│   ├── soutenance/            # Documents de la soutenance du 16 octobre : dossier (Word, PDF), diaporama, fiche technique V1/V2</t>
+          <t>│   ├── soutenance/            # Documents de la soutenance du 16 octobre : dossier (Word, PDF) et diaporama</t>
         </is>
       </c>
     </row>
@@ -1047,7 +1047,7 @@
     <row r="45" ht="43.5" customHeight="1">
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>dictionnaire.md (les données), rgpd.md (les traitements), arborescence.md (ce plan), issue_tree.md et le classeur PPMT_Arborescence_Issue_Tree_V2.xlsx. Le sous-dossier soutenance/ contient les documents de la soutenance du 16 octobre : dossier (Word et PDF), diaporama et fiche technique V1/V2. Les documents de la V1 ont été rangés hors du dépôt, dans _archive/.</t>
+          <t>dictionnaire.md (les données), rgpd.md (les traitements), arborescence.md (ce plan), issue_tree.md et le classeur PPMT_Arborescence_Issue_Tree_V2.xlsx. Le sous-dossier soutenance/ contient les documents de la soutenance du 16 octobre : dossier (Word et PDF) et diaporama. Les documents de la V1 ont été rangés hors du dépôt, dans _archive/.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout validation externe Marché du travail (hors pipeline) + mise à jour README et arborescence
</commit_message>
<xml_diff>
--- a/docs/PPMT_Arborescence_Issue_Tree_V2.xlsx
+++ b/docs/PPMT_Arborescence_Issue_Tree_V2.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B3:B54"/>
+  <dimension ref="B3:B55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -622,229 +622,236 @@
     <row r="22">
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>│   └── ml_tests.py            # ML V2 : classification « en tension » (XGBoost, AUC 0,886)</t>
+          <t>│   ├── ml_tests.py            # ML V2 : classification « en tension » (XGBoost, AUC 0,886)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>│</t>
+          <t>│   └── validation_marche_travail.py  # Validation externe : compare l'indice à l'API Marché du travail (hors pipeline)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>├── src/                       # Le cœur logique : scripts Python permanents du pipeline (ex-« sources/ »)</t>
+          <t>│</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>│   ├── collect.py             # C1 : France Travail (OAuth2, cascade), Adzuna, contours et communes IDF</t>
+          <t>├── src/                       # Le cœur logique : scripts Python permanents du pipeline (ex-« sources/ »)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>│   ├── prepare.py             # C2/C3 : nettoyage, dédoublonnage, salaires, codes ROME, RGPD</t>
+          <t>│   ├── collect.py             # C1 : France Travail (OAuth2, cascade), Adzuna, contours et communes IDF</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>│   └── store.py               # C4 : schéma SQLite, chargement, agrégation SQL, purge 12 mois</t>
+          <t>│   ├── prepare.py             # C2/C3 : nettoyage, dédoublonnage, salaires, codes ROME, RGPD</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>│</t>
+          <t>│   └── store.py               # C4 : schéma SQLite, chargement, agrégation SQL, purge 12 mois</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>├── api/</t>
+          <t>│</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>│   ├── main.py                # C5 : API REST FastAPI (7 routes, clé X-API-Key, Swagger)</t>
+          <t>├── api/</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>│   └── requirements-api.txt   # Dépendances de l'API seule (image Docker allégée)</t>
+          <t>│   ├── main.py                # C5 : API REST FastAPI (7 routes, clé X-API-Key, Swagger)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>│</t>
+          <t>│   └── requirements-api.txt   # Dépendances de l'API seule (image Docker allégée)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>├── webapp/                    # Interface utilisateur (ce que le jury manipule)</t>
+          <t>│</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>│   ├── app.py                 # Dashboard Streamlit : 6 onglets, lit data/ppmt.db</t>
+          <t>├── webapp/                    # Interface utilisateur (ce que le jury manipule)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>│   └── models/                # Modèles ML sauvegardés, utilisés par le dashboard</t>
+          <t>│   ├── app.py                 # Dashboard Streamlit : 6 onglets, lit data/ppmt.db</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>│</t>
+          <t>│   └── models/                # Modèles ML sauvegardés, utilisés par le dashboard</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>├── tests/</t>
+          <t>│</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>│   └── test_pipeline.py       # 57 tests pytest (collecte simulée, règles, base, API)</t>
+          <t>├── tests/</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>│</t>
+          <t>│   └── test_pipeline.py       # 57 tests pytest (collecte simulée, règles, base, API)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>├── docs/</t>
+          <t>│</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>│   ├── soutenance/            # Documents de la soutenance du 16 octobre : dossier (Word, PDF) et diaporama</t>
+          <t>├── docs/</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>│   ├── dictionnaire.md        # Dictionnaire de données</t>
+          <t>│   ├── soutenance/            # Documents de la soutenance du 16 octobre : dossier (Word, PDF) et diaporama</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>│   ├── rgpd.md                # Registre des traitements RGPD</t>
+          <t>│   ├── dictionnaire.md        # Dictionnaire de données</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>│   ├── arborescence.md        # Ce plan commenté</t>
+          <t>│   ├── rgpd.md                # Registre des traitements RGPD</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>│   ├── issue_tree.md          # Issue Tree du projet</t>
+          <t>│   ├── arborescence.md        # Ce plan commenté</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>│   └── PPMT_Arborescence_Issue_Tree_V2.xlsx   # Classeur de cadrage (arborescence, explications, Issue Tree)</t>
+          <t>│   ├── issue_tree.md          # Issue Tree du projet</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>│</t>
+          <t>│   └── PPMT_Arborescence_Issue_Tree_V2.xlsx   # Classeur de cadrage (arborescence, explications, Issue Tree)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>├── run_pipeline.py            # Orchestrateur C1 → C4 (python run_pipeline.py --collect)</t>
+          <t>│</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>├── Dockerfile                 # Image de l'API</t>
+          <t>├── run_pipeline.py            # Orchestrateur C1 → C4 (python run_pipeline.py --collect)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>├── .env.example               # Noms des variables d'environnement (jamais de valeurs)</t>
+          <t>├── Dockerfile                 # Image de l'API</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>├── .gitignore                 # Ignore .env, data/raw/, _archive/, caches Python et pytest, .vscode/</t>
+          <t>├── .env.example               # Noms des variables d'environnement (jamais de valeurs)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>├── pytest.ini                 # Réglages de pytest : dossier des tests, cache rangé dans zz_pytest_cache/</t>
+          <t>├── .gitignore                 # Ignore .env, data/raw/, _archive/, caches Python et pytest, .vscode/</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>├── requirements.txt           # Outils Python à installer (pip install -r requirements.txt)</t>
+          <t>├── pytest.ini                 # Réglages de pytest : dossier des tests, cache rangé dans zz_pytest_cache/</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>├── requirements.txt           # Outils Python à installer (pip install -r requirements.txt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>└── README.md                  # Page d'accueil GitHub : notice, Issue Tree, dictionnaire de données</t>
         </is>
@@ -862,7 +869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B3:B69"/>
+  <dimension ref="B3:B71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -953,190 +960,197 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="70.5" customHeight="1">
+    <row r="24" ht="57" customHeight="1">
       <c r="B24" s="5" t="inlineStr">
         <is>
+          <t>validation_marche_travail.py : le script de validation externe de l'indice. Il interroge l'API « Marché du travail » de France Travail (indicateur officiel de tension, offres et demandeurs par métier) et compare l'indice de PPMT à ces données. Il est séparé du pipeline : il ouvre la base en lecture seule et n'est pas couvert par les 57 tests. Résultat du 8 octobre 2026 : corrélation de rang de +0,09 avec la tension officielle sur 1 301 métiers, +0,89 avec le nombre d'offres de France Travail (l'indice suit le volume d'offres).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="70.5" customHeight="1">
+      <c r="B26" s="5" t="inlineStr">
+        <is>
           <t>Comment sont construites les prédictions : la cible est « indice de tension &gt; 100 » (46 % des 717 métiers) ; les variables d'entrée décrivent le profil des offres du métier (parts de CDI, CDD et intérim, salaire, part de salaires non affichés, expérience demandée, part d'offres pour débutants, longueur des descriptions, famille ROME), sans aucune variable de volume. Chaque probabilité de predictions_tension.csv (colonne proba_tension) est prédite en validation croisée à 5 plis : le métier est prédit par un modèle qui ne l'a pas vu à l'entraînement. Sans la longueur des descriptions, l'AUC de XGBoost passe de 0,886 à 0,795.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="B26" s="4" t="inlineStr">
+    <row r="28" ht="22" customHeight="1">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>🛠️ 4. Le dossier src/ : les machines automatisées de l'usine</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="B27" s="5" t="inlineStr">
+    <row r="29" ht="30" customHeight="1">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>C'est le dossier le plus important pour l'évaluation du bloc (le pipeline). Ce sont des scripts Python permanents, chacun testable et exécutable seul. Il remplace le dossier « sources/ » du plan de mai : même rôle, nom plus courant.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="57" customHeight="1">
-      <c r="B29" s="5" t="inlineStr">
+    <row r="31" ht="57" customHeight="1">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>collect.py (la pompe à API) : se connecte à France Travail en OAuth2 (client_credentials), renouvelle le jeton toutes les 20 minutes, et télécharge les offres. L'API plafonne à 3 150 offres par requête : la collecte découpe en cascade (département, fenêtres de dates, type de contrat). Il lit aussi Adzuna (échantillon de 12 500 offres sur 220 238), les contours des départements et les 1 276 communes d'Île-de-France. 3 tentatives avec attente croissante, pause de 100 ms entre deux appels.</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="43.5" customHeight="1">
-      <c r="B31" s="5" t="inlineStr">
+    <row r="33" ht="43.5" customHeight="1">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>prepare.py (le centre de tri) : prend les fichiers de data/raw/, supprime les doublons (URL, puis titre + entreprise + lieu), complète les salaires manquants par une médiane (56 % non affichés), rattache les offres Adzuna aux codes ROME, harmonise les contrats en 7 catégories, masque les e-mails et téléphones (RGPD).</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="B33" s="5" t="inlineStr">
+    <row r="35" ht="30" customHeight="1">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>store.py (le rangement) : crée le schéma SQLite (4 tables, clés étrangères, contraintes CHECK/UNIQUE, 6 index), charge les offres, calcule les indicateurs de tension en SQL, purge les offres de plus de 12 mois. C'est l'équivalent du schema_db.sql du plan de mai.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="22" customHeight="1">
-      <c r="B35" s="4" t="inlineStr">
+    <row r="37" ht="22" customHeight="1">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>🌐 5. Le dossier api/ : la porte d'entrée pour les développeurs</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="43.5" customHeight="1">
-      <c r="B36" s="5" t="inlineStr">
+    <row r="38" ht="43.5" customHeight="1">
+      <c r="B38" s="5" t="inlineStr">
         <is>
           <t>main.py : l'API FastAPI. requirements-api.txt liste ses seules dépendances, pour une image Docker légère. 7 routes en lecture seule, protégées par une clé X-API-Key (403 sans clé), paramètres validés par Pydantic (422), SQL paramétré, base ouverte en lecture seule. La documentation interactive (Swagger) est sur /docs.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="22" customHeight="1">
-      <c r="B38" s="4" t="inlineStr">
+    <row r="40" ht="22" customHeight="1">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>💻 6. Le dossier webapp/ : la vitrine du magasin</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="43.5" customHeight="1">
-      <c r="B39" s="5" t="inlineStr">
+    <row r="41" ht="43.5" customHeight="1">
+      <c r="B41" s="5" t="inlineStr">
         <is>
           <t>app.py : le dashboard Streamlit (6 onglets, filtres par département, contrat et secteur). Il ne collecte rien : il lit uniquement data/ppmt.db. models/ contient les modèles ML sauvegardés. Une version en ligne sert de secours : https://ppmt-claire.streamlit.app (branche demo-cloud).</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="22" customHeight="1">
-      <c r="B41" s="4" t="inlineStr">
+    <row r="43" ht="22" customHeight="1">
+      <c r="B43" s="4" t="inlineStr">
         <is>
           <t>✅ 7. Le dossier tests/ : le contrôle qualité</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="30" customHeight="1">
-      <c r="B42" s="5" t="inlineStr">
+    <row r="44" ht="30" customHeight="1">
+      <c r="B44" s="5" t="inlineStr">
         <is>
           <t>test_pipeline.py : 57 tests pytest. 4 pour la collecte (API simulées), 31 pour les règles de préparation, 13 pour la base, 9 pour l'API. Limite connue : la cascade France Travail n'a pas encore de test unitaire dédié.</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="22" customHeight="1">
-      <c r="B44" s="4" t="inlineStr">
+    <row r="46" ht="22" customHeight="1">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>📚 8. Le dossier docs/ : la documentation</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="43.5" customHeight="1">
-      <c r="B45" s="5" t="inlineStr">
+    <row r="47" ht="43.5" customHeight="1">
+      <c r="B47" s="5" t="inlineStr">
         <is>
           <t>dictionnaire.md (les données), rgpd.md (les traitements), arborescence.md (ce plan), issue_tree.md et le classeur PPMT_Arborescence_Issue_Tree_V2.xlsx. Le sous-dossier soutenance/ contient les documents de la soutenance du 16 octobre : dossier (Word et PDF) et diaporama. Les documents de la V1 ont été rangés hors du dépôt, dans _archive/.</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="22" customHeight="1">
-      <c r="B47" s="4" t="inlineStr">
+    <row r="49" ht="22" customHeight="1">
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <t>📄 9. Les fichiers à la racine (les indispensables de gestion)</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1">
-      <c r="B48" s="5" t="inlineStr">
+    <row r="50" ht="16.5" customHeight="1">
+      <c r="B50" s="5" t="inlineStr">
         <is>
           <t>README.md : la notice du projet : problème, Issue Tree, arborescence, dictionnaire de données, lancement, API, limites.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="30" customHeight="1">
-      <c r="B50" s="5" t="inlineStr">
-        <is>
-          <t>pytest.ini : les réglages de pytest, l'outil qui lance les 57 tests. Il indique où sont les tests (tests/) et range le cache de pytest dans zz_pytest_cache/, un dossier ignoré par Git qui s'affiche en bas de l'explorateur. Il suffit alors de taper pytest -q.</t>
         </is>
       </c>
     </row>
     <row r="52" ht="30" customHeight="1">
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>requirements.txt : la liste des outils Python. Une seule commande (pip install -r requirements.txt) installe les mêmes versions chez tout le monde.</t>
+          <t>pytest.ini : les réglages de pytest, l'outil qui lance les 57 tests. Il indique où sont les tests (tests/) et range le cache de pytest dans zz_pytest_cache/, un dossier ignoré par Git qui s'affiche en bas de l'explorateur. Il suffit alors de taper pytest -q.</t>
         </is>
       </c>
     </row>
     <row r="54" ht="30" customHeight="1">
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>.env.example : la liste des variables d'environnement attendues (identifiants France Travail et Adzuna), sans aucune valeur. On le copie en .env, qui n'est jamais envoyé sur Git.</t>
+          <t>requirements.txt : la liste des outils Python. Une seule commande (pip install -r requirements.txt) installe les mêmes versions chez tout le monde.</t>
         </is>
       </c>
     </row>
     <row r="56" ht="30" customHeight="1">
       <c r="B56" s="5" t="inlineStr">
         <is>
+          <t>.env.example : la liste des variables d'environnement attendues (identifiants France Travail et Adzuna), sans aucune valeur. On le copie en .env, qui n'est jamais envoyé sur Git.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="30" customHeight="1">
+      <c r="B58" s="5" t="inlineStr">
+        <is>
           <t>run_pipeline.py : l'orchestrateur. Il enchaîne la collecte, la préparation et le stockage ; sans l'option --collect, il repart des fichiers bruts déjà présents dans data/raw/.</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="16.5" customHeight="1">
-      <c r="B58" s="5" t="inlineStr">
+    <row r="60" ht="16.5" customHeight="1">
+      <c r="B60" s="5" t="inlineStr">
         <is>
           <t>Dockerfile : l'image de l'API (FastAPI, Uvicorn et Pydantic seulement), déployable sur Google Cloud Run ou Render.</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="22" customHeight="1">
-      <c r="B60" s="4" t="inlineStr">
+    <row r="62" ht="22" customHeight="1">
+      <c r="B62" s="4" t="inlineStr">
         <is>
           <t>💡 En résumé, comment les données circulent dans cette structure :</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="16.5" customHeight="1">
-      <c r="B61" s="5" t="inlineStr">
-        <is>
-          <t>1. collect.py télécharge les données dans data/raw/ (et écrit son journal dans logs/).</t>
         </is>
       </c>
     </row>
     <row r="63" ht="16.5" customHeight="1">
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>2. prepare.py nettoie le tout et écrit data/processed/offres_unifiees.csv.</t>
+          <t>1. collect.py télécharge les données dans data/raw/ (et écrit son journal dans logs/).</t>
         </is>
       </c>
     </row>
     <row r="65" ht="16.5" customHeight="1">
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>3. store.py range les offres dans la base SQLite data/ppmt.db et calcule les indicateurs de tension.</t>
+          <t>2. prepare.py nettoie le tout et écrit data/processed/offres_unifiees.csv.</t>
         </is>
       </c>
     </row>
     <row r="67" ht="16.5" customHeight="1">
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>4. api/main.py et webapp/app.py lisent cette base : l'API pour les développeurs, le dashboard pour les utilisateurs.</t>
+          <t>3. store.py range les offres dans la base SQLite data/ppmt.db et calcule les indicateurs de tension.</t>
         </is>
       </c>
     </row>
     <row r="69" ht="16.5" customHeight="1">
       <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>4. api/main.py et webapp/app.py lisent cette base : l'API pour les développeurs, le dashboard pour les utilisateurs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="16.5" customHeight="1">
+      <c r="B71" s="5" t="inlineStr">
         <is>
           <t>5. tests/ vérifie chaque étape ; notebook/ml_tests.py ajoute le modèle de classification des métiers en tension.</t>
         </is>
@@ -1154,7 +1168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:C12"/>
+  <dimension ref="A2:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1346,6 +1360,23 @@
       <c r="C12" s="7" t="inlineStr">
         <is>
           <t>Expérimentation ML de la V2</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>(absent)</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>notebook/validation_marche_travail.py</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Validation externe de l'indice (API Marché du travail), hors pipeline</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Issue tree : ajout de la branche Vérifier (validation externe, contrôles de cohérence)
</commit_message>
<xml_diff>
--- a/docs/PPMT_Arborescence_Issue_Tree_V2.xlsx
+++ b/docs/PPMT_Arborescence_Issue_Tree_V2.xlsx
@@ -1392,7 +1392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B3:B30"/>
+  <dimension ref="B3:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1570,28 +1570,49 @@
     <row r="27">
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>└─► 4. METTRE À DISPOSITION (C5) ──┬─► [CLAIRE] Comment l'exposer ? (API FastAPI, 7 routes, clé API)</t>
+          <t>├─► 4. METTRE À DISPOSITION (C5) ──┬─► [CLAIRE] Comment l'exposer ? (API FastAPI, 7 routes, clé API)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    (Pour qui ?)                   ├─► [CLAIRE] Comment le montrer ? (dashboard Streamlit, 6 onglets)</t>
+          <t>│   (Pour qui ?)                   ├─► [CLAIRE] Comment le montrer ? (dashboard Streamlit, 6 onglets)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                                   ├─► [CLAIRE] Comment le garantir ? (57 tests pytest)</t>
+          <t>│                                  ├─► [CLAIRE] Comment le garantir ? (57 tests pytest)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                                   └─► [CLAIRE] Quels métiers sont en tension ? (ML : XGBoost, AUC 0,886)</t>
+          <t>│                                  └─► [CLAIRE] Quels métiers sont en tension ? (ML : XGBoost, AUC 0,886)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>└─► 5. VÉRIFIER (hors pipeline) ───┬─► [CLAIRE] La base est-elle cohérente ? (62 435 offres, 0 doublon, indice moyen 99,99)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    (L'indice est-il fiable ?)     └─► [CLAIRE] Que dit la tension officielle ? (API Marché du travail : ρ = +0,09 ; l'indice suit le volume d'offres)</t>
         </is>
       </c>
     </row>
@@ -1607,7 +1628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B3:B41"/>
+  <dimension ref="B3:B46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1855,35 +1876,70 @@
     <row r="37">
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>└─► 4. METTRE À DISPOSITION (chaîne C5)</t>
+          <t>├─► 4. METTRE À DISPOSITION (chaîne C5)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─► [Claire] API FastAPI : 7 routes, clé X-API-Key (403), validation Pydantic (422), Docker</t>
+          <t>│   ├─► [Claire] API FastAPI : 7 routes, clé X-API-Key (403), validation Pydantic (422), Docker</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─► [Claire] Dashboard Streamlit : 6 onglets, version en ligne de secours</t>
+          <t>│   ├─► [Claire] Dashboard Streamlit : 6 onglets, version en ligne de secours</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─► [Claire] 57 tests pytest : API simulées, règles, base, API</t>
+          <t>│   ├─► [Claire] 57 tests pytest : API simulées, règles, base, API</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─► [Claire · ML] Métiers « en tension » : XGBoost, AUC 0,886 (V1 : fuite de données corrigée)</t>
+          <t>│   └─► [Claire · ML] Métiers « en tension » : XGBoost, AUC 0,886 (V1 : fuite de données corrigée)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>└─► 5. VÉRIFIER (hors pipeline, notebook/validation_marche_travail.py)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─► [Claire] Contrôles de cohérence de la base : 62 435 offres, 0 doublon, 1 514 métiers, indice moyen 99,99</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─► [Claire] Comparaison à la tension officielle (API Marché du travail, 130 métiers) : ρ = +0,09</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─► [Claire] Lecture : l'indice mesure la demande des employeurs (volume d'offres, ρ = +0,89), pas la difficulté à recruter</t>
         </is>
       </c>
     </row>

</xml_diff>